<commit_message>
Ajout du rappel de renouvellement du certificat SSL
</commit_message>
<xml_diff>
--- a/radar-unseen/evenements.xlsx
+++ b/radar-unseen/evenements.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,6 +571,27 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Renouvellement certificat SSL unseenconciergerie.com</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46367</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>